<commit_message>
FEAT: mudando modelo de IA e melhorando extração e classificação de elementos
</commit_message>
<xml_diff>
--- a/app/backend/src/templates/saida/memorial_preenchido.xlsx
+++ b/app/backend/src/templates/saida/memorial_preenchido.xlsx
@@ -1352,7 +1352,7 @@
     <row r="1" ht="14.15" customHeight="1" s="134">
       <c r="B1" s="135" t="inlineStr">
         <is>
-          <t>Teste</t>
+          <t>Test</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1584,7 @@
       <c r="C8" s="140" t="n"/>
       <c r="D8" s="141" t="n"/>
       <c r="E8" s="148" t="n">
-        <v>216.28</v>
+        <v>23.89</v>
       </c>
       <c r="F8" s="148" t="n"/>
       <c r="G8" s="148" t="n">
@@ -1603,10 +1603,14 @@
         </is>
       </c>
       <c r="K8" s="148" t="n">
-        <v>42.07</v>
-      </c>
-      <c r="L8" s="148" t="n"/>
-      <c r="M8" s="152" t="n"/>
+        <v>3.84</v>
+      </c>
+      <c r="L8" s="148" t="n">
+        <v>71.68000000000001</v>
+      </c>
+      <c r="M8" s="152" t="n">
+        <v>63.61</v>
+      </c>
       <c r="N8" s="153">
         <f>K8*L8</f>
         <v/>
@@ -1648,8 +1652,12 @@
       <c r="K9" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="148" t="n"/>
-      <c r="M9" s="152" t="n"/>
+      <c r="L9" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N9" s="153">
         <f>K9*L9</f>
         <v/>
@@ -1691,8 +1699,12 @@
       <c r="K10" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L10" s="148" t="n"/>
-      <c r="M10" s="152" t="n"/>
+      <c r="L10" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N10" s="153">
         <f>K10*L10</f>
         <v/>
@@ -1734,8 +1746,12 @@
       <c r="K11" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="148" t="n"/>
-      <c r="M11" s="152" t="n"/>
+      <c r="L11" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N11" s="153">
         <f>K11*L11</f>
         <v/>
@@ -1777,8 +1793,12 @@
       <c r="K12" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="148" t="n"/>
-      <c r="M12" s="152" t="n"/>
+      <c r="L12" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N12" s="153">
         <f>K12*L12</f>
         <v/>
@@ -1820,8 +1840,12 @@
       <c r="K13" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="148" t="n"/>
-      <c r="M13" s="152" t="n"/>
+      <c r="L13" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N13" s="153">
         <f>K13*L13</f>
         <v/>
@@ -1861,8 +1885,12 @@
       <c r="K14" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L14" s="148" t="n"/>
-      <c r="M14" s="152" t="n"/>
+      <c r="L14" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N14" s="153">
         <f>K14*L14</f>
         <v/>
@@ -1902,8 +1930,12 @@
       <c r="K15" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L15" s="148" t="n"/>
-      <c r="M15" s="152" t="n"/>
+      <c r="L15" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N15" s="153">
         <f>K15*L15</f>
         <v/>
@@ -1943,8 +1975,12 @@
       <c r="K16" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L16" s="148" t="n"/>
-      <c r="M16" s="152" t="n"/>
+      <c r="L16" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N16" s="153">
         <f>K16*L16</f>
         <v/>
@@ -1984,8 +2020,12 @@
       <c r="K17" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L17" s="148" t="n"/>
-      <c r="M17" s="152" t="n"/>
+      <c r="L17" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N17" s="153">
         <f>K17*L17</f>
         <v/>
@@ -2025,8 +2065,12 @@
       <c r="K18" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L18" s="148" t="n"/>
-      <c r="M18" s="152" t="n"/>
+      <c r="L18" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N18" s="153">
         <f>K18*L18</f>
         <v/>
@@ -2066,8 +2110,12 @@
       <c r="K19" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L19" s="148" t="n"/>
-      <c r="M19" s="152" t="n"/>
+      <c r="L19" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N19" s="153">
         <f>K19*L19</f>
         <v/>
@@ -2107,8 +2155,12 @@
       <c r="K20" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L20" s="148" t="n"/>
-      <c r="M20" s="152" t="n"/>
+      <c r="L20" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N20" s="153">
         <f>K20*L20</f>
         <v/>
@@ -2148,8 +2200,12 @@
       <c r="K21" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L21" s="148" t="n"/>
-      <c r="M21" s="152" t="n"/>
+      <c r="L21" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N21" s="153">
         <f>K21*L21</f>
         <v/>
@@ -2189,8 +2245,12 @@
       <c r="K22" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L22" s="148" t="n"/>
-      <c r="M22" s="152" t="n"/>
+      <c r="L22" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N22" s="153">
         <f>K22*L22</f>
         <v/>
@@ -2230,8 +2290,12 @@
       <c r="K23" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L23" s="148" t="n"/>
-      <c r="M23" s="152" t="n"/>
+      <c r="L23" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N23" s="153">
         <f>K23*L23</f>
         <v/>
@@ -2271,8 +2335,12 @@
       <c r="K24" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L24" s="148" t="n"/>
-      <c r="M24" s="152" t="n"/>
+      <c r="L24" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N24" s="153">
         <f>K24*L24</f>
         <v/>
@@ -2312,8 +2380,12 @@
       <c r="K25" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L25" s="148" t="n"/>
-      <c r="M25" s="152" t="n"/>
+      <c r="L25" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N25" s="153">
         <f>K25*L25</f>
         <v/>
@@ -2353,8 +2425,12 @@
       <c r="K26" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L26" s="148" t="n"/>
-      <c r="M26" s="152" t="n"/>
+      <c r="L26" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N26" s="153">
         <f>K26*L26</f>
         <v/>
@@ -2394,8 +2470,12 @@
       <c r="K27" s="148" t="n">
         <v>0</v>
       </c>
-      <c r="L27" s="148" t="n"/>
-      <c r="M27" s="152" t="n"/>
+      <c r="L27" s="148" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="152" t="n">
+        <v>0</v>
+      </c>
       <c r="N27" s="153">
         <f>K27*L27</f>
         <v/>

</xml_diff>